<commit_message>
Version base datos FINAL
</commit_message>
<xml_diff>
--- a/Documents/caapd-facturacion/escritorio/Base de datos/PADRON_MES_2026-10.xlsx
+++ b/Documents/caapd-facturacion/escritorio/Base de datos/PADRON_MES_2026-10.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15 09:11:04</t>
+          <t>2026-10-15 10:10:50</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="19" customWidth="1" min="19" max="19"/>
     <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="24" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="26" customWidth="1" min="23" max="23"/>
     <col width="19" customWidth="1" min="24" max="24"/>
@@ -903,7 +903,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr"/>
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
           <t>000527</t>
@@ -927,8 +931,12 @@
       <c r="F4" s="11" t="n">
         <v>118</v>
       </c>
-      <c r="G4" s="11" t="n"/>
-      <c r="H4" s="11" t="inlineStr"/>
+      <c r="G4" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>82</v>
+      </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -966,12 +974,12 @@
       </c>
       <c r="T4" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U4" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V4" s="14" t="inlineStr">
@@ -984,7 +992,9 @@
           <t>6.0,17.0,10.0,9.0,9.0</t>
         </is>
       </c>
-      <c r="X4" s="14" t="n"/>
+      <c r="X4" s="14" t="n">
+        <v>82</v>
+      </c>
       <c r="Y4" s="14" t="n"/>
       <c r="Z4" s="14" t="n"/>
       <c r="AA4" s="14" t="n"/>
@@ -996,7 +1006,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr"/>
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
           <t>000528</t>
@@ -1020,8 +1034,12 @@
       <c r="F5" s="11" t="n">
         <v>961</v>
       </c>
-      <c r="G5" s="11" t="n"/>
-      <c r="H5" s="11" t="inlineStr"/>
+      <c r="G5" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>39</v>
+      </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -1059,12 +1077,12 @@
       </c>
       <c r="T5" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U5" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V5" s="14" t="inlineStr">
@@ -1077,7 +1095,9 @@
           <t>7.0,16.0,17.0,14.0,7.0</t>
         </is>
       </c>
-      <c r="X5" s="14" t="n"/>
+      <c r="X5" s="14" t="n">
+        <v>39</v>
+      </c>
       <c r="Y5" s="14" t="n"/>
       <c r="Z5" s="14" t="n"/>
       <c r="AA5" s="14" t="n"/>
@@ -1089,7 +1109,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr"/>
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
           <t>000529</t>
@@ -1113,8 +1137,12 @@
       <c r="F6" s="11" t="n">
         <v>258</v>
       </c>
-      <c r="G6" s="11" t="n"/>
-      <c r="H6" s="11" t="inlineStr"/>
+      <c r="G6" s="11" t="n">
+        <v>300</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>42</v>
+      </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -1152,12 +1180,12 @@
       </c>
       <c r="T6" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U6" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V6" s="14" t="inlineStr">
@@ -1170,7 +1198,9 @@
           <t>6.0,6.0,7.0,9.0,9.0</t>
         </is>
       </c>
-      <c r="X6" s="14" t="n"/>
+      <c r="X6" s="14" t="n">
+        <v>42</v>
+      </c>
       <c r="Y6" s="14" t="n"/>
       <c r="Z6" s="14" t="n"/>
       <c r="AA6" s="14" t="n"/>
@@ -1182,7 +1212,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr"/>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
           <t>000530</t>
@@ -1206,8 +1240,12 @@
       <c r="F7" s="11" t="n">
         <v>254</v>
       </c>
-      <c r="G7" s="11" t="n"/>
-      <c r="H7" s="11" t="inlineStr"/>
+      <c r="G7" s="11" t="n">
+        <v>350</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>96</v>
+      </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -1245,12 +1283,12 @@
       </c>
       <c r="T7" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U7" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V7" s="14" t="inlineStr">
@@ -1263,7 +1301,9 @@
           <t>6.0,14.0,9.0,17.0,16.0</t>
         </is>
       </c>
-      <c r="X7" s="14" t="n"/>
+      <c r="X7" s="14" t="n">
+        <v>96</v>
+      </c>
       <c r="Y7" s="14" t="n"/>
       <c r="Z7" s="14" t="n"/>
       <c r="AA7" s="14" t="n"/>
@@ -1275,7 +1315,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr"/>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
           <t>000531</t>
@@ -1299,8 +1343,12 @@
       <c r="F8" s="11" t="n">
         <v>488</v>
       </c>
-      <c r="G8" s="11" t="n"/>
-      <c r="H8" s="11" t="inlineStr"/>
+      <c r="G8" s="11" t="n">
+        <v>488</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -1338,12 +1386,12 @@
       </c>
       <c r="T8" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U8" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V8" s="14" t="inlineStr">
@@ -1356,7 +1404,9 @@
           <t>12.0,9.0,13.0,15.0,10.0</t>
         </is>
       </c>
-      <c r="X8" s="14" t="n"/>
+      <c r="X8" s="14" t="n">
+        <v>0</v>
+      </c>
       <c r="Y8" s="14" t="n"/>
       <c r="Z8" s="14" t="n"/>
       <c r="AA8" s="14" t="n"/>
@@ -1389,7 +1439,7 @@
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="19" customWidth="1" min="12" max="12"/>
@@ -1401,7 +1451,7 @@
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="19" customWidth="1" min="19" max="19"/>
     <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="28" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="26" customWidth="1" min="23" max="23"/>
     <col width="19" customWidth="1" min="24" max="24"/>
@@ -1568,7 +1618,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr"/>
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
           <t>000704</t>
@@ -1592,8 +1646,12 @@
       <c r="F4" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="G4" s="11" t="n"/>
-      <c r="H4" s="11" t="inlineStr"/>
+      <c r="G4" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>7</v>
+      </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -1631,12 +1689,12 @@
       </c>
       <c r="T4" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U4" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V4" s="14" t="inlineStr">
@@ -1649,7 +1707,9 @@
           <t>18.0,18.0,0.0,8.0,13.0</t>
         </is>
       </c>
-      <c r="X4" s="14" t="n"/>
+      <c r="X4" s="14" t="n">
+        <v>7</v>
+      </c>
       <c r="Y4" s="14" t="n"/>
       <c r="Z4" s="14" t="n"/>
       <c r="AA4" s="14" t="n"/>
@@ -1661,7 +1721,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr"/>
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
           <t>000534</t>
@@ -1685,8 +1749,12 @@
       <c r="F5" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="G5" s="11" t="n"/>
-      <c r="H5" s="11" t="inlineStr"/>
+      <c r="G5" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>5</v>
+      </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -1724,12 +1792,12 @@
       </c>
       <c r="T5" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U5" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V5" s="14" t="inlineStr">
@@ -1742,7 +1810,9 @@
           <t>10.0,8.0,9.0,105.0,18.0</t>
         </is>
       </c>
-      <c r="X5" s="14" t="n"/>
+      <c r="X5" s="14" t="n">
+        <v>5</v>
+      </c>
       <c r="Y5" s="14" t="n"/>
       <c r="Z5" s="14" t="n"/>
       <c r="AA5" s="14" t="n"/>
@@ -1754,7 +1824,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr"/>
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
           <t>000533</t>
@@ -1778,11 +1852,15 @@
       <c r="F6" s="11" t="n">
         <v>557</v>
       </c>
-      <c r="G6" s="11" t="n"/>
-      <c r="H6" s="11" t="inlineStr"/>
+      <c r="G6" s="11" t="n">
+        <v>854</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>297</v>
+      </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>MEDIDOR_DANADO</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr"/>
@@ -1817,12 +1895,12 @@
       </c>
       <c r="T6" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U6" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V6" s="14" t="inlineStr">
@@ -1835,7 +1913,9 @@
           <t>7.0,12.0,7.0,11.0,11.0</t>
         </is>
       </c>
-      <c r="X6" s="14" t="n"/>
+      <c r="X6" s="14" t="n">
+        <v>297</v>
+      </c>
       <c r="Y6" s="14" t="n"/>
       <c r="Z6" s="14" t="n"/>
       <c r="AA6" s="14" t="n"/>
@@ -1847,7 +1927,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr"/>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
           <t>000536</t>
@@ -1871,8 +1955,12 @@
       <c r="F7" s="11" t="n">
         <v>333</v>
       </c>
-      <c r="G7" s="11" t="n"/>
-      <c r="H7" s="11" t="inlineStr"/>
+      <c r="G7" s="11" t="n">
+        <v>400</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>67</v>
+      </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -1910,12 +1998,12 @@
       </c>
       <c r="T7" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U7" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V7" s="14" t="inlineStr">
@@ -1928,7 +2016,9 @@
           <t>18.0,6.0,17.0,13.0,14.0</t>
         </is>
       </c>
-      <c r="X7" s="14" t="n"/>
+      <c r="X7" s="14" t="n">
+        <v>67</v>
+      </c>
       <c r="Y7" s="14" t="n"/>
       <c r="Z7" s="14" t="n"/>
       <c r="AA7" s="14" t="n"/>
@@ -1961,7 +2051,7 @@
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="19" customWidth="1" min="12" max="12"/>
@@ -1973,7 +2063,7 @@
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="19" customWidth="1" min="19" max="19"/>
     <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="28" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="27" customWidth="1" min="23" max="23"/>
     <col width="19" customWidth="1" min="24" max="24"/>
@@ -2140,7 +2230,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr"/>
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
           <t>000498</t>
@@ -2164,8 +2258,12 @@
       <c r="F4" s="11" t="n">
         <v>249</v>
       </c>
-      <c r="G4" s="11" t="n"/>
-      <c r="H4" s="11" t="inlineStr"/>
+      <c r="G4" s="11" t="n">
+        <v>312</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>63</v>
+      </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -2203,12 +2301,12 @@
       </c>
       <c r="T4" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U4" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V4" s="14" t="inlineStr">
@@ -2221,7 +2319,9 @@
           <t>7.0,14.0,10.0,16.0,15.0</t>
         </is>
       </c>
-      <c r="X4" s="14" t="n"/>
+      <c r="X4" s="14" t="n">
+        <v>63</v>
+      </c>
       <c r="Y4" s="14" t="n"/>
       <c r="Z4" s="14" t="n"/>
       <c r="AA4" s="14" t="n"/>
@@ -2233,7 +2333,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr"/>
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
           <t>000308</t>
@@ -2257,8 +2361,12 @@
       <c r="F5" s="11" t="n">
         <v>137</v>
       </c>
-      <c r="G5" s="11" t="n"/>
-      <c r="H5" s="11" t="inlineStr"/>
+      <c r="G5" s="11" t="n">
+        <v>140</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -2296,12 +2404,12 @@
       </c>
       <c r="T5" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U5" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V5" s="14" t="inlineStr">
@@ -2314,7 +2422,9 @@
           <t>19.0,24.0,16.0,13.0,28.0</t>
         </is>
       </c>
-      <c r="X5" s="14" t="n"/>
+      <c r="X5" s="14" t="n">
+        <v>13</v>
+      </c>
       <c r="Y5" s="14" t="n"/>
       <c r="Z5" s="14" t="n"/>
       <c r="AA5" s="14" t="n"/>
@@ -2326,7 +2436,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr"/>
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
           <t>000308</t>
@@ -2350,11 +2464,15 @@
       <c r="F6" s="11" t="n">
         <v>745</v>
       </c>
-      <c r="G6" s="11" t="n"/>
-      <c r="H6" s="11" t="inlineStr"/>
+      <c r="G6" s="11" t="n">
+        <v>755</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>10</v>
+      </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>LECTURA_ESTIMADA</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr"/>
@@ -2379,12 +2497,12 @@
       </c>
       <c r="T6" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U6" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V6" s="14" t="inlineStr"/>
@@ -2397,7 +2515,11 @@
       <c r="AC6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr"/>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
           <t>000274</t>
@@ -2421,8 +2543,12 @@
       <c r="F7" s="11" t="n">
         <v>503</v>
       </c>
-      <c r="G7" s="11" t="n"/>
-      <c r="H7" s="11" t="inlineStr"/>
+      <c r="G7" s="11" t="n">
+        <v>521</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>18</v>
+      </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -2460,12 +2586,12 @@
       </c>
       <c r="T7" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U7" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V7" s="14" t="inlineStr">
@@ -2478,7 +2604,9 @@
           <t>16.0,11.0,8.0,11.0,11.0</t>
         </is>
       </c>
-      <c r="X7" s="14" t="n"/>
+      <c r="X7" s="14" t="n">
+        <v>18</v>
+      </c>
       <c r="Y7" s="14" t="n"/>
       <c r="Z7" s="14" t="n"/>
       <c r="AA7" s="14" t="n"/>
@@ -2490,7 +2618,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr"/>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
           <t>000746</t>
@@ -2514,8 +2646,12 @@
       <c r="F8" s="11" t="n">
         <v>384</v>
       </c>
-      <c r="G8" s="11" t="n"/>
-      <c r="H8" s="11" t="inlineStr"/>
+      <c r="G8" s="11" t="n">
+        <v>398</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>14</v>
+      </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -2553,12 +2689,12 @@
       </c>
       <c r="T8" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U8" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V8" s="14" t="inlineStr">
@@ -2571,7 +2707,9 @@
           <t>10.0,17.0,16.0,16.0,7.0</t>
         </is>
       </c>
-      <c r="X8" s="14" t="n"/>
+      <c r="X8" s="14" t="n">
+        <v>14</v>
+      </c>
       <c r="Y8" s="14" t="n"/>
       <c r="Z8" s="14" t="n"/>
       <c r="AA8" s="14" t="n"/>
@@ -2583,7 +2721,11 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr"/>
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
           <t>000850</t>
@@ -2607,8 +2749,12 @@
       <c r="F9" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="G9" s="11" t="n"/>
-      <c r="H9" s="11" t="inlineStr"/>
+      <c r="G9" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>28</v>
+      </c>
       <c r="I9" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -2646,12 +2792,12 @@
       </c>
       <c r="T9" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U9" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V9" s="14" t="inlineStr">
@@ -2664,7 +2810,9 @@
           <t>12.0</t>
         </is>
       </c>
-      <c r="X9" s="14" t="n"/>
+      <c r="X9" s="14" t="n">
+        <v>28</v>
+      </c>
       <c r="Y9" s="14" t="n"/>
       <c r="Z9" s="14" t="n"/>
       <c r="AA9" s="14" t="n"/>
@@ -2697,7 +2845,7 @@
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="19" customWidth="1" min="12" max="12"/>
@@ -2709,7 +2857,7 @@
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="19" customWidth="1" min="19" max="19"/>
     <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="28" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="26" customWidth="1" min="23" max="23"/>
     <col width="19" customWidth="1" min="24" max="24"/>
@@ -2876,7 +3024,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr"/>
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
           <t>000002</t>
@@ -2900,8 +3052,12 @@
       <c r="F4" s="11" t="n">
         <v>367</v>
       </c>
-      <c r="G4" s="11" t="n"/>
-      <c r="H4" s="11" t="inlineStr"/>
+      <c r="G4" s="11" t="n">
+        <v>370</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -2939,12 +3095,12 @@
       </c>
       <c r="T4" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U4" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V4" s="14" t="inlineStr">
@@ -2957,7 +3113,9 @@
           <t>8.0,14.0,17.0,9.0,8.0</t>
         </is>
       </c>
-      <c r="X4" s="14" t="n"/>
+      <c r="X4" s="14" t="n">
+        <v>3</v>
+      </c>
       <c r="Y4" s="14" t="n"/>
       <c r="Z4" s="14" t="n"/>
       <c r="AA4" s="14" t="n"/>
@@ -2969,7 +3127,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr"/>
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
           <t>000004</t>
@@ -2993,11 +3155,15 @@
       <c r="F5" s="11" t="n">
         <v>609</v>
       </c>
-      <c r="G5" s="11" t="n"/>
-      <c r="H5" s="11" t="inlineStr"/>
+      <c r="G5" s="11" t="n">
+        <v>610</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>MEDIDOR_DANADO</t>
         </is>
       </c>
       <c r="J5" s="11" t="inlineStr"/>
@@ -3032,12 +3198,12 @@
       </c>
       <c r="T5" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U5" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V5" s="14" t="inlineStr">
@@ -3050,7 +3216,9 @@
           <t>10.0,16.0,17.0,14.0,9.0</t>
         </is>
       </c>
-      <c r="X5" s="14" t="n"/>
+      <c r="X5" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="Y5" s="14" t="n"/>
       <c r="Z5" s="14" t="n"/>
       <c r="AA5" s="14" t="n"/>
@@ -3062,7 +3230,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr"/>
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
           <t>000006</t>
@@ -3086,11 +3258,15 @@
       <c r="F6" s="11" t="n">
         <v>559</v>
       </c>
-      <c r="G6" s="11" t="n"/>
-      <c r="H6" s="11" t="inlineStr"/>
+      <c r="G6" s="11" t="n">
+        <v>565</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>6</v>
+      </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>LECTURA_ESTIMADA</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr"/>
@@ -3125,12 +3301,12 @@
       </c>
       <c r="T6" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U6" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V6" s="14" t="inlineStr">
@@ -3143,7 +3319,9 @@
           <t>18.0,18.0,6.0,9.0,6.0</t>
         </is>
       </c>
-      <c r="X6" s="14" t="n"/>
+      <c r="X6" s="14" t="n">
+        <v>6</v>
+      </c>
       <c r="Y6" s="14" t="n"/>
       <c r="Z6" s="14" t="n"/>
       <c r="AA6" s="14" t="n"/>
@@ -3155,7 +3333,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr"/>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
           <t>000007</t>
@@ -3179,11 +3361,15 @@
       <c r="F7" s="11" t="n">
         <v>889</v>
       </c>
-      <c r="G7" s="11" t="n"/>
-      <c r="H7" s="11" t="inlineStr"/>
+      <c r="G7" s="11" t="n">
+        <v>904</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>15</v>
+      </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>LECTURA_ESTIMADA</t>
         </is>
       </c>
       <c r="J7" s="11" t="inlineStr"/>
@@ -3218,12 +3404,12 @@
       </c>
       <c r="T7" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U7" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V7" s="14" t="inlineStr">
@@ -3236,7 +3422,9 @@
           <t>12.0,10.0,7.0,9.0,15.0</t>
         </is>
       </c>
-      <c r="X7" s="14" t="n"/>
+      <c r="X7" s="14" t="n">
+        <v>15</v>
+      </c>
       <c r="Y7" s="14" t="n"/>
       <c r="Z7" s="14" t="n"/>
       <c r="AA7" s="14" t="n"/>
@@ -3248,7 +3436,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr"/>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
           <t>000771</t>
@@ -3272,11 +3464,15 @@
       <c r="F8" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="11" t="n"/>
-      <c r="H8" s="11" t="inlineStr"/>
+      <c r="G8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>LECTURA_ESTIMADA</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr"/>
@@ -3311,12 +3507,12 @@
       </c>
       <c r="T8" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U8" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V8" s="14" t="inlineStr">
@@ -3329,7 +3525,9 @@
           <t>0.0,0.0,0.0,0.0,0.0</t>
         </is>
       </c>
-      <c r="X8" s="14" t="n"/>
+      <c r="X8" s="14" t="n">
+        <v>0</v>
+      </c>
       <c r="Y8" s="14" t="n"/>
       <c r="Z8" s="14" t="n"/>
       <c r="AA8" s="14" t="n"/>
@@ -3362,7 +3560,7 @@
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="19" customWidth="1" min="12" max="12"/>
@@ -3374,7 +3572,7 @@
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="19" customWidth="1" min="19" max="19"/>
     <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="28" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="27" customWidth="1" min="23" max="23"/>
     <col width="19" customWidth="1" min="24" max="24"/>
@@ -3541,7 +3739,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr"/>
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
           <t>000089</t>
@@ -3565,8 +3767,12 @@
       <c r="F4" s="11" t="n">
         <v>485</v>
       </c>
-      <c r="G4" s="11" t="n"/>
-      <c r="H4" s="11" t="inlineStr"/>
+      <c r="G4" s="11" t="n">
+        <v>485</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -3604,12 +3810,12 @@
       </c>
       <c r="T4" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U4" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V4" s="14" t="inlineStr">
@@ -3622,7 +3828,9 @@
           <t>8.0,14.0,13.0,7.0,18.0</t>
         </is>
       </c>
-      <c r="X4" s="14" t="n"/>
+      <c r="X4" s="14" t="n">
+        <v>0</v>
+      </c>
       <c r="Y4" s="14" t="n"/>
       <c r="Z4" s="14" t="n"/>
       <c r="AA4" s="14" t="n"/>
@@ -3634,7 +3842,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr"/>
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
           <t>000092</t>
@@ -3658,8 +3870,12 @@
       <c r="F5" s="11" t="n">
         <v>1741</v>
       </c>
-      <c r="G5" s="11" t="n"/>
-      <c r="H5" s="11" t="inlineStr"/>
+      <c r="G5" s="11" t="n">
+        <v>1743</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -3697,12 +3913,12 @@
       </c>
       <c r="T5" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U5" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V5" s="14" t="inlineStr">
@@ -3715,7 +3931,9 @@
           <t>9.0,16.0,13.0,12.0,16.0</t>
         </is>
       </c>
-      <c r="X5" s="14" t="n"/>
+      <c r="X5" s="14" t="n">
+        <v>2</v>
+      </c>
       <c r="Y5" s="14" t="n"/>
       <c r="Z5" s="14" t="n"/>
       <c r="AA5" s="14" t="n"/>
@@ -3727,7 +3945,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr"/>
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
           <t>000095</t>
@@ -3751,8 +3973,12 @@
       <c r="F6" s="11" t="n">
         <v>875</v>
       </c>
-      <c r="G6" s="11" t="n"/>
-      <c r="H6" s="11" t="inlineStr"/>
+      <c r="G6" s="11" t="n">
+        <v>958</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>83</v>
+      </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -3790,12 +4016,12 @@
       </c>
       <c r="T6" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U6" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V6" s="14" t="inlineStr">
@@ -3808,7 +4034,9 @@
           <t>8.0,16.0,8.0,18.0,16.0</t>
         </is>
       </c>
-      <c r="X6" s="14" t="n"/>
+      <c r="X6" s="14" t="n">
+        <v>83</v>
+      </c>
       <c r="Y6" s="14" t="n"/>
       <c r="Z6" s="14" t="n"/>
       <c r="AA6" s="14" t="n"/>
@@ -3820,7 +4048,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr"/>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
           <t>000098</t>
@@ -3844,11 +4076,15 @@
       <c r="F7" s="11" t="n">
         <v>1063</v>
       </c>
-      <c r="G7" s="11" t="n"/>
-      <c r="H7" s="11" t="inlineStr"/>
+      <c r="G7" s="11" t="n">
+        <v>1075</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>12</v>
+      </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>LECTURA_ESTIMADA</t>
         </is>
       </c>
       <c r="J7" s="11" t="inlineStr"/>
@@ -3883,12 +4119,12 @@
       </c>
       <c r="T7" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U7" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V7" s="14" t="inlineStr">
@@ -3901,7 +4137,9 @@
           <t>10.0,8.0,9.0,17.0,14.0</t>
         </is>
       </c>
-      <c r="X7" s="14" t="n"/>
+      <c r="X7" s="14" t="n">
+        <v>12</v>
+      </c>
       <c r="Y7" s="14" t="n"/>
       <c r="Z7" s="14" t="n"/>
       <c r="AA7" s="14" t="n"/>
@@ -3913,7 +4151,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr"/>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
           <t>000099</t>
@@ -3937,11 +4179,15 @@
       <c r="F8" s="11" t="n">
         <v>1499</v>
       </c>
-      <c r="G8" s="11" t="n"/>
-      <c r="H8" s="11" t="inlineStr"/>
+      <c r="G8" s="11" t="n">
+        <v>1511</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>12</v>
+      </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>LECTURA_ESTIMADA</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr"/>
@@ -3976,12 +4222,12 @@
       </c>
       <c r="T8" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U8" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>bryanlaricoro28@gmail.com</t>
         </is>
       </c>
       <c r="V8" s="14" t="inlineStr">
@@ -3994,7 +4240,9 @@
           <t>17.0,15.0,12.0,15.0,12.0</t>
         </is>
       </c>
-      <c r="X8" s="14" t="n"/>
+      <c r="X8" s="14" t="n">
+        <v>12</v>
+      </c>
       <c r="Y8" s="14" t="n"/>
       <c r="Z8" s="14" t="n"/>
       <c r="AA8" s="14" t="n"/>
@@ -4027,8 +4275,8 @@
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="19" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
@@ -4039,7 +4287,7 @@
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="19" customWidth="1" min="19" max="19"/>
     <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="24" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="27" customWidth="1" min="23" max="23"/>
     <col width="19" customWidth="1" min="24" max="24"/>
@@ -4206,7 +4454,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr"/>
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
           <t>000055</t>
@@ -4230,14 +4482,22 @@
       <c r="F4" s="11" t="n">
         <v>486</v>
       </c>
-      <c r="G4" s="11" t="n"/>
-      <c r="H4" s="11" t="inlineStr"/>
+      <c r="G4" s="11" t="n">
+        <v>586</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>100</v>
+      </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="J4" s="11" t="inlineStr"/>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>todo bom</t>
+        </is>
+      </c>
       <c r="K4" s="11" t="inlineStr"/>
       <c r="L4" s="12" t="n">
         <v>0</v>
@@ -4269,12 +4529,12 @@
       </c>
       <c r="T4" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U4" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V4" s="14" t="inlineStr">
@@ -4287,7 +4547,9 @@
           <t>7.0,12.0,12.0,15.0,13.0</t>
         </is>
       </c>
-      <c r="X4" s="14" t="n"/>
+      <c r="X4" s="14" t="n">
+        <v>100</v>
+      </c>
       <c r="Y4" s="14" t="n"/>
       <c r="Z4" s="14" t="n"/>
       <c r="AA4" s="14" t="n"/>
@@ -4299,7 +4561,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr"/>
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
           <t>000066</t>
@@ -4323,8 +4589,12 @@
       <c r="F5" s="11" t="n">
         <v>520</v>
       </c>
-      <c r="G5" s="11" t="n"/>
-      <c r="H5" s="11" t="inlineStr"/>
+      <c r="G5" s="11" t="n">
+        <v>540</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>20</v>
+      </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
           <t>NORMAL</t>
@@ -4362,12 +4632,12 @@
       </c>
       <c r="T5" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U5" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V5" s="14" t="inlineStr">
@@ -4380,7 +4650,9 @@
           <t>14.0,6.0,16.0,17.0,7.0</t>
         </is>
       </c>
-      <c r="X5" s="14" t="n"/>
+      <c r="X5" s="14" t="n">
+        <v>20</v>
+      </c>
       <c r="Y5" s="14" t="n"/>
       <c r="Z5" s="14" t="n"/>
       <c r="AA5" s="14" t="n"/>
@@ -4392,7 +4664,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr"/>
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
           <t>000059</t>
@@ -4416,14 +4692,22 @@
       <c r="F6" s="11" t="n">
         <v>1571</v>
       </c>
-      <c r="G6" s="11" t="n"/>
-      <c r="H6" s="11" t="inlineStr"/>
+      <c r="G6" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>429</v>
+      </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="J6" s="11" t="inlineStr"/>
+          <t>FUGA_VISIBLE</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>hay fuga</t>
+        </is>
+      </c>
       <c r="K6" s="11" t="inlineStr"/>
       <c r="L6" s="12" t="n">
         <v>0</v>
@@ -4455,12 +4739,12 @@
       </c>
       <c r="T6" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U6" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V6" s="14" t="inlineStr">
@@ -4473,7 +4757,9 @@
           <t>18.0,10.0,18.0,16.0,11.0</t>
         </is>
       </c>
-      <c r="X6" s="14" t="n"/>
+      <c r="X6" s="14" t="n">
+        <v>429</v>
+      </c>
       <c r="Y6" s="14" t="n"/>
       <c r="Z6" s="14" t="n"/>
       <c r="AA6" s="14" t="n"/>
@@ -4485,7 +4771,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr"/>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
           <t>000061</t>
@@ -4509,11 +4799,15 @@
       <c r="F7" s="11" t="n">
         <v>141</v>
       </c>
-      <c r="G7" s="11" t="n"/>
-      <c r="H7" s="11" t="inlineStr"/>
+      <c r="G7" s="11" t="n">
+        <v>635</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>494</v>
+      </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>MEDIDOR_EMPANADO</t>
         </is>
       </c>
       <c r="J7" s="11" t="inlineStr"/>
@@ -4548,12 +4842,12 @@
       </c>
       <c r="T7" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U7" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V7" s="14" t="inlineStr">
@@ -4566,7 +4860,9 @@
           <t>12.0,8.0,13.0,6.0,17.0</t>
         </is>
       </c>
-      <c r="X7" s="14" t="n"/>
+      <c r="X7" s="14" t="n">
+        <v>494</v>
+      </c>
       <c r="Y7" s="14" t="n"/>
       <c r="Z7" s="14" t="n"/>
       <c r="AA7" s="14" t="n"/>
@@ -4578,7 +4874,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr"/>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
           <t>000070</t>
@@ -4602,11 +4902,15 @@
       <c r="F8" s="11" t="n">
         <v>671</v>
       </c>
-      <c r="G8" s="11" t="n"/>
-      <c r="H8" s="11" t="inlineStr"/>
+      <c r="G8" s="11" t="n">
+        <v>741</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>70</v>
+      </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>MEDIDOR_DANADO</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr"/>
@@ -4641,12 +4945,12 @@
       </c>
       <c r="T8" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U8" s="14" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>andresore28@gmail.com</t>
         </is>
       </c>
       <c r="V8" s="14" t="inlineStr">
@@ -4659,7 +4963,9 @@
           <t>14.0,18.0,8.0,14.0,7.0</t>
         </is>
       </c>
-      <c r="X8" s="14" t="n"/>
+      <c r="X8" s="14" t="n">
+        <v>70</v>
+      </c>
       <c r="Y8" s="14" t="n"/>
       <c r="Z8" s="14" t="n"/>
       <c r="AA8" s="14" t="n"/>
@@ -6125,7 +6431,8 @@
     "fecha_emision": "2026-10-15",
     "fecha_vencimiento": "2026-10-30"
   },
-  "ultimo_envio_lectores": "2026-10-15 07:54:19"
+  "ultimo_envio_lectores": "2026-10-15 07:54:19",
+  "ultima_descarga_lectores": "2026-10-15 10:00:55"
 }</t>
         </is>
       </c>

</xml_diff>

<commit_message>
(feat): Se arreglo el bug de creacion de usuarios nuevos y se arreglo los colores de los botones de filtros
</commit_message>
<xml_diff>
--- a/Documents/caapd-facturacion/escritorio/Base de datos/PADRON_MES_2026-10.xlsx
+++ b/Documents/caapd-facturacion/escritorio/Base de datos/PADRON_MES_2026-10.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15 17:09:17</t>
+          <t>2026-10-16 16:56:27</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10">
@@ -634,7 +634,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11">
@@ -655,7 +655,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>29_719.00</t>
+          <t>32_719.00</t>
         </is>
       </c>
     </row>
@@ -713,14 +713,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC8"/>
+  <dimension ref="A1:AC13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="37" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
@@ -732,7 +732,7 @@
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="19" customWidth="1" min="19" max="19"/>
     <col width="17" customWidth="1" min="20" max="20"/>
@@ -1092,26 +1092,26 @@
       <c r="A6" s="11" t="inlineStr"/>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>000529</t>
+          <t>000714</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>220014925</t>
+          <t>2148715</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>SURCO VILLENA, SUSY BETTY</t>
+          <t>FERNANDEZ ROSPIGLUIOSI ANDREA</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>AYACUCHO S/N</t>
+          <t>MARAÑON 112</t>
         </is>
       </c>
       <c r="F6" s="11" t="n">
-        <v>258</v>
+        <v>0</v>
       </c>
       <c r="G6" s="11" t="n"/>
       <c r="H6" s="11" t="inlineStr"/>
@@ -1123,13 +1123,13 @@
       <c r="J6" s="11" t="inlineStr"/>
       <c r="K6" s="11" t="inlineStr"/>
       <c r="L6" s="12" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="M6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N6" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O6" s="13" t="inlineStr">
         <is>
@@ -1139,17 +1139,11 @@
       <c r="P6" s="11" t="inlineStr"/>
       <c r="Q6" s="14" t="inlineStr">
         <is>
-          <t>30770890</t>
-        </is>
-      </c>
-      <c r="R6" s="14" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="S6" s="14" t="n">
-        <v>9</v>
-      </c>
+          <t>111111111111</t>
+        </is>
+      </c>
+      <c r="R6" s="14" t="inlineStr"/>
+      <c r="S6" s="14" t="n"/>
       <c r="T6" s="14" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
@@ -1165,46 +1159,38 @@
           <t>A</t>
         </is>
       </c>
-      <c r="W6" s="14" t="inlineStr">
-        <is>
-          <t>6.0,6.0,7.0,9.0,9.0</t>
-        </is>
-      </c>
+      <c r="W6" s="14" t="inlineStr"/>
       <c r="X6" s="14" t="n"/>
       <c r="Y6" s="14" t="n"/>
       <c r="Z6" s="14" t="n"/>
       <c r="AA6" s="14" t="n"/>
-      <c r="AB6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC6" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="AB6" s="14" t="n"/>
+      <c r="AC6" s="14" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr"/>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>000530</t>
+          <t>000714</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>6563926</t>
+          <t>3321881</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>TORRES COA, CILA CAMILA</t>
+          <t>FERNANDEZ ROSPIGLUIOSI ANDREA</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>AYACUCHO S/N</t>
+          <t>MARAÑON 112</t>
         </is>
       </c>
       <c r="F7" s="11" t="n">
-        <v>254</v>
+        <v>0</v>
       </c>
       <c r="G7" s="11" t="n"/>
       <c r="H7" s="11" t="inlineStr"/>
@@ -1215,34 +1201,18 @@
       </c>
       <c r="J7" s="11" t="inlineStr"/>
       <c r="K7" s="11" t="inlineStr"/>
-      <c r="L7" s="12" t="n">
-        <v>182</v>
-      </c>
-      <c r="M7" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="O7" s="13" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="L7" s="11" t="inlineStr"/>
+      <c r="M7" s="11" t="inlineStr"/>
+      <c r="N7" s="11" t="inlineStr"/>
+      <c r="O7" s="11" t="inlineStr"/>
       <c r="P7" s="11" t="inlineStr"/>
       <c r="Q7" s="14" t="inlineStr">
         <is>
-          <t>30770036</t>
-        </is>
-      </c>
-      <c r="R7" s="14" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="S7" s="14" t="n">
-        <v>16</v>
-      </c>
+          <t>111111111111</t>
+        </is>
+      </c>
+      <c r="R7" s="14" t="inlineStr"/>
+      <c r="S7" s="14" t="n"/>
       <c r="T7" s="14" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
@@ -1253,52 +1223,34 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="V7" s="14" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="W7" s="14" t="inlineStr">
-        <is>
-          <t>6.0,14.0,9.0,17.0,16.0</t>
-        </is>
-      </c>
-      <c r="X7" s="14" t="n"/>
-      <c r="Y7" s="14" t="n"/>
-      <c r="Z7" s="14" t="n"/>
-      <c r="AA7" s="14" t="n"/>
-      <c r="AB7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC7" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="V7" s="14" t="inlineStr"/>
+      <c r="W7" s="14" t="inlineStr"/>
+      <c r="X7" s="14" t="inlineStr"/>
+      <c r="Y7" s="14" t="inlineStr"/>
+      <c r="Z7" s="14" t="inlineStr"/>
+      <c r="AA7" s="14" t="inlineStr"/>
+      <c r="AB7" s="14" t="inlineStr"/>
+      <c r="AC7" s="14" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr"/>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>000531</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>6563939</t>
-        </is>
-      </c>
+          <t>000851</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr"/>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>TORRES HUAMANI, AMELIA BENITA</t>
+          <t>ORE SOTO ANDRES</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>AYACUCHO S/N</t>
-        </is>
-      </c>
-      <c r="F8" s="11" t="n">
-        <v>488</v>
-      </c>
+          <t>CALLE ROBLES</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="n"/>
       <c r="G8" s="11" t="n"/>
       <c r="H8" s="11" t="inlineStr"/>
       <c r="I8" s="11" t="inlineStr">
@@ -1325,20 +1277,14 @@
       <c r="P8" s="11" t="inlineStr"/>
       <c r="Q8" s="14" t="inlineStr">
         <is>
-          <t>30778043</t>
-        </is>
-      </c>
-      <c r="R8" s="14" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="S8" s="14" t="n">
-        <v>10</v>
-      </c>
+          <t>93258763</t>
+        </is>
+      </c>
+      <c r="R8" s="14" t="inlineStr"/>
+      <c r="S8" s="14" t="n"/>
       <c r="T8" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>LEIDO</t>
         </is>
       </c>
       <c r="U8" s="14" t="inlineStr">
@@ -1351,19 +1297,434 @@
           <t>A</t>
         </is>
       </c>
-      <c r="W8" s="14" t="inlineStr">
-        <is>
-          <t>12.0,9.0,13.0,15.0,10.0</t>
-        </is>
-      </c>
+      <c r="W8" s="14" t="inlineStr"/>
       <c r="X8" s="14" t="n"/>
       <c r="Y8" s="14" t="n"/>
       <c r="Z8" s="14" t="n"/>
       <c r="AA8" s="14" t="n"/>
-      <c r="AB8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC8" s="14" t="n">
+      <c r="AB8" s="14" t="n"/>
+      <c r="AC8" s="14" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr"/>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>000852</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>16984112</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>PROBANDO ANDO PRUEBA1</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>CALLE LOS SUEÑOS</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="11" t="inlineStr"/>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr"/>
+      <c r="K9" s="11" t="inlineStr"/>
+      <c r="L9" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="P9" s="11" t="inlineStr"/>
+      <c r="Q9" s="14" t="inlineStr">
+        <is>
+          <t>11111154711</t>
+        </is>
+      </c>
+      <c r="R9" s="14" t="inlineStr"/>
+      <c r="S9" s="14" t="n"/>
+      <c r="T9" s="14" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="U9" s="14" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="V9" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="W9" s="14" t="inlineStr"/>
+      <c r="X9" s="14" t="n"/>
+      <c r="Y9" s="14" t="n"/>
+      <c r="Z9" s="14" t="n"/>
+      <c r="AA9" s="14" t="n"/>
+      <c r="AB9" s="14" t="n"/>
+      <c r="AC9" s="14" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr"/>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>000852</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>3219810</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>PROBANDO ANDO PRUEBA1</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>CALLE LOS SUEÑOS</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="11" t="inlineStr"/>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr"/>
+      <c r="K10" s="11" t="inlineStr"/>
+      <c r="L10" s="11" t="inlineStr"/>
+      <c r="M10" s="11" t="inlineStr"/>
+      <c r="N10" s="11" t="inlineStr"/>
+      <c r="O10" s="11" t="inlineStr"/>
+      <c r="P10" s="11" t="inlineStr"/>
+      <c r="Q10" s="14" t="inlineStr">
+        <is>
+          <t>11111154711</t>
+        </is>
+      </c>
+      <c r="R10" s="14" t="inlineStr"/>
+      <c r="S10" s="14" t="n"/>
+      <c r="T10" s="14" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="U10" s="14" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="V10" s="14" t="inlineStr"/>
+      <c r="W10" s="14" t="inlineStr"/>
+      <c r="X10" s="14" t="inlineStr"/>
+      <c r="Y10" s="14" t="inlineStr"/>
+      <c r="Z10" s="14" t="inlineStr"/>
+      <c r="AA10" s="14" t="inlineStr"/>
+      <c r="AB10" s="14" t="inlineStr"/>
+      <c r="AC10" s="14" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr"/>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>000529</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>220014925</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>SURCO VILLENA, SUSY BETTY</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>AYACUCHO S/N</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>258</v>
+      </c>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="11" t="inlineStr"/>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr"/>
+      <c r="K11" s="11" t="inlineStr"/>
+      <c r="L11" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="O11" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="P11" s="11" t="inlineStr"/>
+      <c r="Q11" s="14" t="inlineStr">
+        <is>
+          <t>30770890</t>
+        </is>
+      </c>
+      <c r="R11" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="S11" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="T11" s="14" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="U11" s="14" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="V11" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="W11" s="14" t="inlineStr">
+        <is>
+          <t>6.0,6.0,7.0,9.0,9.0</t>
+        </is>
+      </c>
+      <c r="X11" s="14" t="n"/>
+      <c r="Y11" s="14" t="n"/>
+      <c r="Z11" s="14" t="n"/>
+      <c r="AA11" s="14" t="n"/>
+      <c r="AB11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC11" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr"/>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>000530</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>6563926</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>TORRES COA, CILA CAMILA</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>AYACUCHO S/N</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>254</v>
+      </c>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="11" t="inlineStr"/>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="J12" s="11" t="inlineStr"/>
+      <c r="K12" s="11" t="inlineStr"/>
+      <c r="L12" s="12" t="n">
+        <v>182</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="O12" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="P12" s="11" t="inlineStr"/>
+      <c r="Q12" s="14" t="inlineStr">
+        <is>
+          <t>30770036</t>
+        </is>
+      </c>
+      <c r="R12" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="S12" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="T12" s="14" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="U12" s="14" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="V12" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="W12" s="14" t="inlineStr">
+        <is>
+          <t>6.0,14.0,9.0,17.0,16.0</t>
+        </is>
+      </c>
+      <c r="X12" s="14" t="n"/>
+      <c r="Y12" s="14" t="n"/>
+      <c r="Z12" s="14" t="n"/>
+      <c r="AA12" s="14" t="n"/>
+      <c r="AB12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr"/>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>000531</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>6563939</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>TORRES HUAMANI, AMELIA BENITA</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>AYACUCHO S/N</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>488</v>
+      </c>
+      <c r="G13" s="11" t="n"/>
+      <c r="H13" s="11" t="inlineStr"/>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="inlineStr"/>
+      <c r="K13" s="11" t="inlineStr"/>
+      <c r="L13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="P13" s="11" t="inlineStr"/>
+      <c r="Q13" s="14" t="inlineStr">
+        <is>
+          <t>30778043</t>
+        </is>
+      </c>
+      <c r="R13" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="S13" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="T13" s="14" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="U13" s="14" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="V13" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="W13" s="14" t="inlineStr">
+        <is>
+          <t>12.0,9.0,13.0,15.0,10.0</t>
+        </is>
+      </c>
+      <c r="X13" s="14" t="n"/>
+      <c r="Y13" s="14" t="n"/>
+      <c r="Z13" s="14" t="n"/>
+      <c r="AA13" s="14" t="n"/>
+      <c r="AB13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1897,7 +2258,11 @@
         </is>
       </c>
       <c r="J7" s="11" t="inlineStr"/>
-      <c r="K7" s="11" t="inlineStr"/>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>000000170</t>
+        </is>
+      </c>
       <c r="L7" s="12" t="n">
         <v>0</v>
       </c>
@@ -1949,9 +2314,15 @@
       <c r="X7" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="Y7" s="14" t="n"/>
-      <c r="Z7" s="14" t="n"/>
-      <c r="AA7" s="14" t="n"/>
+      <c r="Y7" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="Z7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="14" t="n">
+        <v>5</v>
+      </c>
       <c r="AB7" s="14" t="n">
         <v>0</v>
       </c>
@@ -4701,7 +5072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -5649,27 +6020,27 @@
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>12345678</t>
+          <t>111111111111</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>000070</t>
+          <t>000714</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>HUAMANI CASTRO, BERTHA</t>
+          <t>FERNANDEZ ROSPIGLUIOSI ANDREA</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>HUAQUILLO</t>
+          <t>AYACUCHO</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>HUAQUILLO BAJO</t>
+          <t>MARAÑON 112</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
@@ -5684,34 +6055,34 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>6659861</t>
+          <t>2148715,3321881</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>75849301</t>
+          <t>12345678</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>000850</t>
+          <t>000070</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>MAMANI APAZA, CRISTIAN ALFREDO</t>
+          <t>HUAMANI CASTRO, BERTHA</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>BARRIO DE CHAUPI</t>
+          <t>HUAQUILLO</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>CALLE NUEVA 10</t>
+          <t>HUAQUILLO BAJO</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
@@ -5726,34 +6097,34 @@
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>24355999</t>
+          <t>6659861</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>30769321</t>
+          <t>75849301</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>000534</t>
+          <t>000850</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>NEYRA DE USCAMAYTA, MANUELA ANA</t>
+          <t>MAMANI APAZA, CRISTIAN ALFREDO</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>CHAUPICERCA</t>
+          <t>BARRIO DE CHAUPI</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>CHAUPICERCA S/N</t>
+          <t>CALLE NUEVA 10</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
@@ -5768,24 +6139,24 @@
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>6593461</t>
+          <t>24355999</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>30769931-1</t>
+          <t>30769321</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>000533</t>
+          <t>000534</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>ROMERO CHAUCAYANQUI JUSTO MARCELO</t>
+          <t>NEYRA DE USCAMAYTA, MANUELA ANA</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -5810,24 +6181,24 @@
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>6593433</t>
+          <t>6593461</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>30770890</t>
+          <t>93258763</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>000529</t>
+          <t>000851</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>SURCO VILLENA, SUSY BETTY</t>
+          <t>ORE SOTO ANDRES</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
@@ -5837,7 +6208,7 @@
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>AYACUCHO S/N</t>
+          <t>CALLE ROBLES</t>
         </is>
       </c>
       <c r="F29" s="11" t="inlineStr">
@@ -5850,26 +6221,22 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="H29" s="11" t="inlineStr">
-        <is>
-          <t>220014925</t>
-        </is>
-      </c>
+      <c r="H29" s="11" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>30770036</t>
+          <t>11111154711</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>000530</t>
+          <t>000852</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>TORRES COA, CILA CAMILA</t>
+          <t>PROBANDO ANDO PRUEBA1</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -5879,7 +6246,7 @@
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>AYACUCHO S/N</t>
+          <t>CALLE LOS SUEÑOS</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
@@ -5894,34 +6261,34 @@
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>6563926</t>
+          <t>16984112,3219810</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>30778043</t>
+          <t>30769931-1</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>000531</t>
+          <t>000533</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>TORRES HUAMANI, AMELIA BENITA</t>
+          <t>ROMERO CHAUCAYANQUI JUSTO MARCELO</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>AYACUCHO</t>
+          <t>CHAUPICERCA</t>
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>AYACUCHO S/N</t>
+          <t>CHAUPICERCA S/N</t>
         </is>
       </c>
       <c r="F31" s="11" t="inlineStr">
@@ -5936,47 +6303,173 @@
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
-          <t>6563939</t>
+          <t>6593433</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
+          <t>30770890</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>000529</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>SURCO VILLENA, SUSY BETTY</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>AYACUCHO</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>AYACUCHO S/N</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H32" s="11" t="inlineStr">
+        <is>
+          <t>220014925</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>30770036</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>000530</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>TORRES COA, CILA CAMILA</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>AYACUCHO</t>
+        </is>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>AYACUCHO S/N</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H33" s="11" t="inlineStr">
+        <is>
+          <t>6563926</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>30778043</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>000531</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>TORRES HUAMANI, AMELIA BENITA</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>AYACUCHO</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>AYACUCHO S/N</t>
+        </is>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H34" s="11" t="inlineStr">
+        <is>
+          <t>6563939</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
           <t>30769896</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>000536</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>USCAMAYTA NEYRA, DAVID JESUS</t>
         </is>
       </c>
-      <c r="D32" s="11" t="inlineStr">
+      <c r="D35" s="11" t="inlineStr">
         <is>
           <t>CHAUPICERCA</t>
         </is>
       </c>
-      <c r="E32" s="11" t="inlineStr">
+      <c r="E35" s="11" t="inlineStr">
         <is>
           <t>CHAUPICERCA S/N</t>
         </is>
       </c>
-      <c r="F32" s="11" t="inlineStr">
+      <c r="F35" s="11" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G32" s="11" t="inlineStr">
+      <c r="G35" s="11" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="H32" s="11" t="inlineStr">
+      <c r="H35" s="11" t="inlineStr">
         <is>
           <t>6593726</t>
         </is>
@@ -6138,7 +6631,7 @@
     "BARRIO DE PACHAYZA": "lector.pachayza@prueba.local",
     "HUAQUILLO": "lector.huaquillo@prueba.local"
   },
-  "ultimo_recibo": 169,
+  "ultimo_recibo": 170,
   "mes_actual": {
     "periodo": "2026-10",
     "estado": "ABIERTO",
@@ -6155,7 +6648,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5">

</xml_diff>